<commit_message>
Make flat prices editable in the pricing sheet too, and cover all prices
The Flat Price column in data/pricing.xlsx is now authoritative: editing it
changes what buyers are charged (falling back to the app's built-in price if a
row is blank/absent). The per-sqft column still overrides flat when filled.

Also added the previously code-only prices to the sheet so it covers
everything: coffered/tray ceilings (per room) and the 9'/10' ceiling-height
upgrades (per floor). Those are flat-only — their per-sqft cell shows "n/a".

- pricing.ts now returns {flat, perSqft, tbd} per key (readPricing).
- Component resolves price via priceFor()/flatFor(), threaded through category
  options, toggle items, quantity (per-room) items, and per-floor options.
- Verified flat overrides flow through all three shapes; regenerated the sheet
  with the complete row set and refreshed instructions.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pricing.xlsx
+++ b/data/pricing.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Per SqFt Rates" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Prices" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Instructions" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="106">
   <si>
     <t>Option Key (do not edit)</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Option</t>
   </si>
   <si>
-    <t>Current Flat Price ($)</t>
-  </si>
-  <si>
-    <t>Price per Sq Ft ($) — fill in to override</t>
+    <t>Flat Price ($) — edit to change</t>
+  </si>
+  <si>
+    <t>Price per Sq Ft ($) — fill in to scale with house size</t>
   </si>
   <si>
     <t>roof__other-timberline</t>
@@ -131,6 +131,9 @@
     <t>TBD</t>
   </si>
   <si>
+    <t>n/a</t>
+  </si>
+  <si>
     <t>flooring__flooring-stain</t>
   </si>
   <si>
@@ -164,12 +167,39 @@
     <t>Designer Palette — Custom</t>
   </si>
   <si>
+    <t>ceiling-height__9ft</t>
+  </si>
+  <si>
+    <t>Ceiling Height (per floor)</t>
+  </si>
+  <si>
+    <t>9' Ceiling</t>
+  </si>
+  <si>
+    <t>ceiling-height__10ft</t>
+  </si>
+  <si>
+    <t>10' Ceiling</t>
+  </si>
+  <si>
+    <t>ceiling-features__coffered</t>
+  </si>
+  <si>
+    <t>Trim Upgrades</t>
+  </si>
+  <si>
+    <t>Coffered Ceiling (per room)</t>
+  </si>
+  <si>
+    <t>ceiling-features__tray</t>
+  </si>
+  <si>
+    <t>Tray Ceiling with Light Rail (per room)</t>
+  </si>
+  <si>
     <t>ceiling-features__trim-panel-foyer-stairwell</t>
   </si>
   <si>
-    <t>Trim Upgrades</t>
-  </si>
-  <si>
     <t>Trim Panel Package — Foyer Stairwell</t>
   </si>
   <si>
@@ -254,40 +284,49 @@
     <t/>
   </si>
   <si>
-    <t>Fill in the 'Price per Sq Ft' column (the highlighted one) for any option whose price</t>
-  </si>
-  <si>
-    <t>should scale with house size. Leave it blank for options that keep their flat price.</t>
-  </si>
-  <si>
-    <t>When a rate is filled in, the website computes that option's price for each buyer as:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    price = rate x the buyer's house size (sq ft)</t>
-  </si>
-  <si>
-    <t>You enter each buyer's house size on the Builder Dashboard (the password-protected page).</t>
-  </si>
-  <si>
-    <t>If a buyer has no house size entered yet, per-sqft options show 'Price TBD' in their portal.</t>
-  </si>
-  <si>
-    <t>The 'Current Flat Price' column is for reference only — changing it here does NOT change</t>
-  </si>
-  <si>
-    <t>the website. Flat prices live in the app itself; ask to have those changed.</t>
+    <t>This is the single place to set every upgrade price. Two editable columns:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Flat Price — the option's price. Edit it to change what buyers are charged.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Price per Sq Ft — leave blank for a flat price, OR fill it in to make the</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    price scale with house size. When filled, it OVERRIDES the flat price and</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    the website computes:  price = rate x the buyer's house size (sq ft).</t>
+  </si>
+  <si>
+    <t>You enter each buyer's house size on the Builder Dashboard (the password page).</t>
+  </si>
+  <si>
+    <t>If a per-sqft option has no house size entered for a buyer, it shows 'Price TBD'</t>
+  </si>
+  <si>
+    <t>in their portal until you add one.</t>
+  </si>
+  <si>
+    <t>Cells marked 'n/a' in the Price per Sq Ft column are structural or per-room</t>
+  </si>
+  <si>
+    <t>prices (ceiling heights, coffered/tray ceilings) that don't scale with house</t>
+  </si>
+  <si>
+    <t>size — set their Flat Price only.</t>
+  </si>
+  <si>
+    <t>'TBD' in a Flat Price cell means the buyer sees 'Price TBD' (e.g. the custom</t>
+  </si>
+  <si>
+    <t>countertop option). Replace it with a number once a price is known.</t>
   </si>
   <si>
     <t>Do not edit the 'Option Key' column — it's how rows are matched to website options.</t>
   </si>
   <si>
-    <t>Not listed here: ceiling heights (fixed per-floor prices) and the coffered/tray ceilings</t>
-  </si>
-  <si>
-    <t>(priced per room with a quantity picker, not by house size).</t>
-  </si>
-  <si>
-    <t>After saving changes, the file needs to be published (committed and pushed) before the</t>
+    <t>After saving changes, the file must be published (committed and pushed) before the</t>
   </si>
   <si>
     <t>live site picks it up — just ask to 'publish the new pricing'.</t>
@@ -301,7 +340,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -321,6 +360,12 @@
     </font>
     <font>
       <color rgb="FF0000FF"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <i/>
+      <color rgb="FF999999"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -360,15 +405,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,14 +757,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -925,20 +974,22 @@
       <c r="C14" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="4"/>
+      <c r="E14" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D15" s="3">
         <v>500</v>
@@ -947,13 +998,13 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D16" s="3">
         <v>200</v>
@@ -962,13 +1013,13 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D17" s="3">
         <v>450</v>
@@ -977,13 +1028,13 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D18" s="3">
         <v>400</v>
@@ -992,91 +1043,99 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D19" s="3">
-        <v>6400</v>
-      </c>
-      <c r="E19" s="4"/>
+        <v>19850</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D20" s="3">
-        <v>4500</v>
-      </c>
-      <c r="E20" s="4"/>
+        <v>38500</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D21" s="3">
-        <v>4600</v>
-      </c>
-      <c r="E21" s="4"/>
+        <v>6500</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="C22" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D22" s="3">
-        <v>90000</v>
-      </c>
-      <c r="E22" s="4"/>
+        <v>9900</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D23" s="3">
-        <v>110000</v>
+        <v>6400</v>
       </c>
       <c r="E23" s="4"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>64</v>
       </c>
       <c r="D24" s="3">
-        <v>15000</v>
+        <v>4500</v>
       </c>
       <c r="E24" s="4"/>
     </row>
@@ -1085,13 +1144,13 @@
         <v>65</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>66</v>
       </c>
       <c r="D25" s="3">
-        <v>5000</v>
+        <v>4600</v>
       </c>
       <c r="E25" s="4"/>
     </row>
@@ -1100,192 +1159,272 @@
         <v>67</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D26" s="3">
-        <v>25000</v>
+        <v>90000</v>
       </c>
       <c r="E26" s="4"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D27" s="3">
-        <v>7500</v>
+        <v>110000</v>
       </c>
       <c r="E27" s="4"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D28" s="3">
-        <v>16500</v>
+        <v>15000</v>
       </c>
       <c r="E28" s="4"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="C29" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D29" s="3">
-        <v>7500</v>
+        <v>5000</v>
       </c>
       <c r="E29" s="4"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D30" s="3">
+        <v>25000</v>
+      </c>
+      <c r="E30" s="4"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31" s="3">
+        <v>7500</v>
+      </c>
+      <c r="E31" s="4"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D32" s="3">
+        <v>16500</v>
+      </c>
+      <c r="E32" s="4"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D33" s="3">
+        <v>7500</v>
+      </c>
+      <c r="E33" s="4"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D34" s="3">
         <v>12000</v>
       </c>
-      <c r="E30" s="4"/>
+      <c r="E34" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>78</v>
+      <c r="A1" s="7" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>83</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update pricing: per-sqft rates for finishes/insulation, flat bumps on windows & garage doors
Per Sq Ft added: roof other-timberline 1.60, siding other-alside 1.25,
hardieplank-all-sides 18.00, flooring stain 1.40, crown moulding upstairs 1.92,
energy efficiency package 4.00. Flat changes: black windows 850->10000,
black garage doors 300->1000, coachman doors 1200->1800.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pricing.xlsx
+++ b/data/pricing.xlsx
@@ -1,11 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FA812C-1FA1-45E6-A15C-99416334E662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Prices" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Instructions" state="visible" r:id="rId5"/>
+    <sheet name="Prices" sheetId="1" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -335,23 +339,23 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="$#,##0"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="\$#,##0"/>
+    <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -359,14 +363,14 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
+      <sz val="10"/>
       <color rgb="FF999999"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -756,9 +760,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E34"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -767,7 +771,7 @@
     <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -797,7 +801,9 @@
       <c r="D2" s="3">
         <v>400</v>
       </c>
-      <c r="E2" s="4"/>
+      <c r="E2" s="4">
+        <v>1.6</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -812,7 +818,9 @@
       <c r="D3" s="3">
         <v>350</v>
       </c>
-      <c r="E3" s="4"/>
+      <c r="E3" s="4">
+        <v>1.25</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -827,7 +835,9 @@
       <c r="D4" s="3">
         <v>55000</v>
       </c>
-      <c r="E4" s="4"/>
+      <c r="E4" s="4">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -840,7 +850,7 @@
         <v>15</v>
       </c>
       <c r="D5" s="3">
-        <v>850</v>
+        <v>10000</v>
       </c>
       <c r="E5" s="4"/>
     </row>
@@ -915,7 +925,7 @@
         <v>27</v>
       </c>
       <c r="D10" s="3">
-        <v>300</v>
+        <v>1000</v>
       </c>
       <c r="E10" s="4"/>
     </row>
@@ -930,7 +940,7 @@
         <v>29</v>
       </c>
       <c r="D11" s="3">
-        <v>1200</v>
+        <v>1800</v>
       </c>
       <c r="E11" s="4"/>
     </row>
@@ -994,7 +1004,9 @@
       <c r="D15" s="3">
         <v>500</v>
       </c>
-      <c r="E15" s="4"/>
+      <c r="E15" s="4">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
@@ -1152,7 +1164,9 @@
       <c r="D25" s="3">
         <v>4600</v>
       </c>
-      <c r="E25" s="4"/>
+      <c r="E25" s="4">
+        <v>1.92</v>
+      </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -1287,23 +1301,25 @@
       <c r="D34" s="3">
         <v>12000</v>
       </c>
-      <c r="E34" s="4"/>
+      <c r="E34" s="4">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A24"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>88</v>
       </c>
@@ -1425,6 +1441,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Allow per-sqft pricing for ceiling heights
Ceiling-height (9'/10') rows in data/pricing.xlsx are now per-sqft-eligible
(their Price per Sq Ft cell is editable instead of "n/a"). floorLineFor
resolves via priceFor so a rate computes as rate × the buyer's sqft; when a
per-sqft ceiling has no house size entered yet it surfaces as "Price TBD"
throughout — the floor pill, the group subtotal, the header/grand-total
summary, and the review-and-sign modal all handle the TBD case now.
Flat ceiling prices still work when no rate is set.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/pricing.xlsx
+++ b/data/pricing.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FA812C-1FA1-45E6-A15C-99416334E662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
-    <sheet name="Prices" sheetId="1" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="Prices" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Instructions" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="106">
   <si>
     <t>Option Key (do not edit)</t>
   </si>
@@ -339,23 +338,23 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="\$#,##0"/>
-    <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -363,14 +362,8 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF0000FF"/>
       <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF999999"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -418,10 +411,10 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -760,9 +753,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -771,7 +764,7 @@
     <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1066,9 +1059,7 @@
       <c r="D19" s="3">
         <v>19850</v>
       </c>
-      <c r="E19" s="6" t="s">
-        <v>39</v>
-      </c>
+      <c r="E19" s="6"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
@@ -1083,9 +1074,7 @@
       <c r="D20" s="3">
         <v>38500</v>
       </c>
-      <c r="E20" s="6" t="s">
-        <v>39</v>
-      </c>
+      <c r="E20" s="6"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
@@ -1307,19 +1296,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" ht="15.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>88</v>
       </c>
@@ -1441,6 +1430,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>